<commit_message>
update Dictionnaire des données
</commit_message>
<xml_diff>
--- a/ressources/BookHub - Dictionnaire des données.xlsx
+++ b/ressources/BookHub - Dictionnaire des données.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdeparscau2026\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdeparscau2026\Documents\projects\BookHub\ressources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A8BBE9-E499-4058-940A-B02BD99D2D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45303925-02B8-49B1-A1F9-53563FB51D7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5DCC8868-A66B-4C56-BC16-FD1664C4DD1A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="86">
   <si>
     <t>Table</t>
   </si>
@@ -249,13 +249,61 @@
   </si>
   <si>
     <t>idOpinion</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>RETURNED</t>
+  </si>
+  <si>
+    <t>Reservations</t>
+  </si>
+  <si>
+    <t>idReservation</t>
+  </si>
+  <si>
+    <t>Identifiant unique de la réservation</t>
+  </si>
+  <si>
+    <t>rank</t>
+  </si>
+  <si>
+    <t>Rang dans la réservation</t>
+  </si>
+  <si>
+    <t>Commentaire</t>
+  </si>
+  <si>
+    <t>Colonne supprimée pour redondance avec les dates de fin</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>Mot de passe de l'utilisateur</t>
+  </si>
+  <si>
+    <t>Members</t>
+  </si>
+  <si>
+    <t>idMember</t>
+  </si>
+  <si>
+    <t>Identifiant unique de l'adhérent</t>
+  </si>
+  <si>
+    <t>Email de l'adhérent</t>
+  </si>
+  <si>
+    <t>Table pour vérifier l'email des nouveaux comptes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,6 +323,29 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -318,15 +389,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -661,15 +734,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{786D925F-4ADE-41FD-A030-7E456FFC006E}">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
     <col min="4" max="4" width="32.28515625" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="51.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -685,193 +761,206 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="F1" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5" t="s">
+      <c r="F2" s="7"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5" t="s">
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" s="7"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E5" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5" t="s">
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E6" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="C7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E7" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7" t="s">
+      <c r="F7" s="8"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E8" s="5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7" t="s">
+      <c r="F8" s="8"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C9" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E9" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7" t="s">
+      <c r="F9" s="8"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C10" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="7"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7" t="s">
+      <c r="E10" s="5"/>
+      <c r="F10" s="8"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="C11" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E11" s="5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7" t="s">
+      <c r="F11" s="8"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D12" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E12" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7" t="s">
+      <c r="F12" s="8"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="C13" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E13" s="5" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>39</v>
-      </c>
+      <c r="F13" s="8"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="5"/>
       <c r="B14" s="5" t="s">
         <v>40</v>
       </c>
@@ -879,253 +968,406 @@
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E15" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5" t="s">
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C16" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E16" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B17" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="7" t="s">
+      <c r="C17" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E17" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7" t="s">
+      <c r="F17" s="8"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C18" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D18" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E18" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7" t="s">
+      <c r="F18" s="8"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C19" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D19" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E19" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="F19" s="8"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B20" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="5" t="s">
+      <c r="C20" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E20" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5" t="s">
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="5" t="s">
+      <c r="C21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E21" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+      <c r="F21" s="7"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B22" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="7" t="s">
+      <c r="C22" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E22" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7" t="s">
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="7" t="s">
+      <c r="C23" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E22" s="7"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7" t="s">
+      <c r="E23" s="5"/>
+      <c r="F23" s="8"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="5"/>
+      <c r="B24" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C24" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D24" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E23" s="7"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7" t="s">
+      <c r="E24" s="5"/>
+      <c r="F24" s="8"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="5"/>
+      <c r="B25" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="7" t="s">
+      <c r="C25" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E25" s="5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7" t="s">
+      <c r="F25" s="8"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="5"/>
+      <c r="B26" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="7" t="s">
+      <c r="C26" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E26" s="5" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
+      <c r="F26" s="8"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B27" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="5" t="s">
+      <c r="C27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E27" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="2"/>
-      <c r="B27" s="5" t="s">
+      <c r="F27" s="7"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C28" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E28" s="2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="2"/>
-      <c r="B28" s="5" t="s">
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C29" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="2"/>
-      <c r="B29" s="5" t="s">
+      <c r="E29" s="2"/>
+      <c r="F29" s="7"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="6"/>
+      <c r="B30" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E30" s="6"/>
+      <c r="F30" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="2" t="s">
+      <c r="C31" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E31" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="2"/>
-      <c r="B30" s="5" t="s">
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="C32" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E32" s="2" t="s">
         <v>29</v>
       </c>
+      <c r="F32" s="7"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="5"/>
+      <c r="B34" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="5"/>
+      <c r="B35" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F38" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update Dictionnaire des donnees
</commit_message>
<xml_diff>
--- a/ressources/BookHub - Dictionnaire des données.xlsx
+++ b/ressources/BookHub - Dictionnaire des données.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdeparscau2026\Documents\projects\BookHub\ressources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28497330-0639-442E-B9F3-C3E8618C5D9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BB82EEF-1134-4BB3-A419-1A921EF33C8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5DCC8868-A66B-4C56-BC16-FD1664C4DD1A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="100">
   <si>
     <t>Table</t>
   </si>
@@ -104,9 +104,6 @@
     <t>Identifiant unique du livre</t>
   </si>
   <si>
-    <t>Varchar(20)</t>
-  </si>
-  <si>
     <t>Identifiant naturel du livre</t>
   </si>
   <si>
@@ -312,6 +309,36 @@
   </si>
   <si>
     <t>Rôle de l'utilisateur</t>
+  </si>
+  <si>
+    <t>Float</t>
+  </si>
+  <si>
+    <t>Varchar(17)</t>
+  </si>
+  <si>
+    <t>L'ISBN 13 va jusqu'à 13 chiffres et 4 tirets</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>Description du livre</t>
+  </si>
+  <si>
+    <t>TEXT</t>
+  </si>
+  <si>
+    <t>Max 1000 caractères</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>Numéro de téléphone de l'utilisateur</t>
+  </si>
+  <si>
+    <t>De 1 à 5</t>
   </si>
 </sst>
 </file>
@@ -749,13 +776,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{786D925F-4ADE-41FD-A030-7E456FFC006E}">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" customWidth="1"/>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="32.28515625" customWidth="1"/>
+    <col min="4" max="4" width="33.5703125" customWidth="1"/>
     <col min="5" max="5" width="16.5703125" customWidth="1"/>
     <col min="6" max="6" width="51.5703125" customWidth="1"/>
   </cols>
@@ -777,7 +804,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -817,16 +844,16 @@
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F4" s="7"/>
     </row>
@@ -842,71 +869,69 @@
         <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F5" s="7"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>13</v>
+        <v>97</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
+        <v>88</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>51</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="E6" s="2"/>
       <c r="F6" s="7"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="7"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="E8" s="2"/>
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="C9" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>6</v>
-      </c>
-      <c r="F8" s="8"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>8</v>
       </c>
       <c r="F9" s="8"/>
     </row>
@@ -916,503 +941,541 @@
         <v>23</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>7</v>
+        <v>91</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="8"/>
+        <v>8</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="5"/>
+        <v>24</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>50</v>
+      </c>
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
       <c r="B12" s="5" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>29</v>
-      </c>
+        <v>94</v>
+      </c>
+      <c r="E12" s="5"/>
       <c r="F12" s="8"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="5" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>33</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="E13" s="5"/>
       <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="5" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" s="8"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F15" s="8"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="E18" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="7"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2" t="s">
+      <c r="F20" s="8"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" s="7"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="5" t="s">
+      <c r="C21" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E21" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" s="8"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F18" s="8"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E19" s="5" t="s">
+      <c r="F23" s="7"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="8"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F20" s="8"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="E21" s="2" t="s">
+      <c r="E24" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" s="7"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F21" s="7"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F22" s="7"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F23" s="8"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E24" s="5"/>
-      <c r="F24" s="8"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E25" s="5"/>
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="5" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F26" s="8"/>
+        <v>50</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" s="5"/>
+      <c r="F27" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="5"/>
+      <c r="B28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F28" s="8"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="5"/>
+      <c r="B29" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="5" t="s">
+      <c r="C29" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" s="8"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E27" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F27" s="8"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
+      <c r="B30" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C30" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="E30" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F30" s="7"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="2"/>
+      <c r="B31" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F28" s="7"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F29" s="7"/>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2" t="s">
+      <c r="D31" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E30" s="2"/>
-      <c r="F30" s="7"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="6"/>
-      <c r="B31" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E31" s="6"/>
-      <c r="F31" s="9" t="s">
-        <v>78</v>
-      </c>
+      <c r="E31" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F31" s="7"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E32" s="2"/>
+      <c r="F32" s="7"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="6"/>
+      <c r="B33" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E33" s="6"/>
+      <c r="F33" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="7"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F33" s="7"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+      <c r="C34" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F34" s="7"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="2"/>
+      <c r="B35" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F35" s="7"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="C36" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" s="5" t="s">
+      <c r="E36" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F36" s="8"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="4"/>
+      <c r="B37" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E34" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="F34" s="8"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="4"/>
-      <c r="B35" s="5" t="s">
+      <c r="C37" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F35" s="8"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="E36" s="5"/>
-      <c r="F36" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>58</v>
-      </c>
       <c r="E37" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F37" s="8"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
       <c r="B38" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E38" s="5"/>
+      <c r="F38" s="8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="5"/>
+      <c r="B39" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C38" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F38" s="8"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
+      <c r="C40" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="C41" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D39" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E39" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F40" s="7"/>
+      <c r="E42" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F42" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>